<commit_message>
corellation, statistics, override resolved
</commit_message>
<xml_diff>
--- a/data/processed/model_avg_F1.xlsx
+++ b/data/processed/model_avg_F1.xlsx
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8868817090988159</v>
+        <v>0.8868817061912723</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8846564118455096</v>
+        <v>0.8846564103917378</v>
       </c>
     </row>
     <row r="4">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8840566713635515</v>
+        <v>0.8840566742710951</v>
       </c>
     </row>
     <row r="6">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.5549715815520868</v>
+        <v>0.5549715800983149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>